<commit_message>
Draft essential feature bank system
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Feature.xlsx
+++ b/C/Project/ATM_Sim/Doc/Feature.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499AD89F-BFC8-4EFE-8296-643CC686A7C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04BC374-A224-4627-A545-0B88E85D7FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feature" sheetId="1" r:id="rId1"/>
+    <sheet name="ATM" sheetId="1" r:id="rId1"/>
+    <sheet name="Bank system" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="44">
   <si>
     <t>Feature</t>
   </si>
@@ -103,6 +104,60 @@
   </si>
   <si>
     <t>Allow the user to cancel a transaction before it is completed</t>
+  </si>
+  <si>
+    <t>Navigation (main menu)</t>
+  </si>
+  <si>
+    <t>Display after validation of the PIN. Allow the user selects options in ATM</t>
+  </si>
+  <si>
+    <t>Transaction Processing</t>
+  </si>
+  <si>
+    <t>Withdrawl Processing</t>
+  </si>
+  <si>
+    <t>Deposit Processing</t>
+  </si>
+  <si>
+    <t>Transaction History</t>
+  </si>
+  <si>
+    <t>Account Authentication</t>
+  </si>
+  <si>
+    <t>Account Management</t>
+  </si>
+  <si>
+    <t>Balance Management</t>
+  </si>
+  <si>
+    <t>Verify the user's account/PIN when required</t>
+  </si>
+  <si>
+    <t>Manage user account information and status</t>
+  </si>
+  <si>
+    <t>Store and update the customer's account balance</t>
+  </si>
+  <si>
+    <t>Process transactions and received from the ATM</t>
+  </si>
+  <si>
+    <t>Deduct the withdrawn amount from the user's account</t>
+  </si>
+  <si>
+    <t>Add the deposited amount the user's account</t>
+  </si>
+  <si>
+    <t>Provide the latest account balance to the ATM</t>
+  </si>
+  <si>
+    <t>Record completed transactions for the account</t>
+  </si>
+  <si>
+    <t>Need confirm</t>
   </si>
 </sst>
 </file>
@@ -434,7 +489,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24" style="2" customWidth="1"/>
@@ -546,8 +601,106 @@
         <v>14</v>
       </c>
     </row>
+    <row r="14" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D76FD108-D374-497F-925F-3F73DFCAD246}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24.90625" customWidth="1"/>
+    <col min="2" max="2" width="52.36328125" customWidth="1"/>
+    <col min="3" max="3" width="39.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refined the name feature in the Feature file
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Feature.xlsx
+++ b/C/Project/ATM_Sim/Doc/Feature.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499AD89F-BFC8-4EFE-8296-643CC686A7C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BF85B32-D4AA-4139-BEE5-D6FD82369E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feature" sheetId="1" r:id="rId1"/>
+    <sheet name="ATM" sheetId="1" r:id="rId1"/>
+    <sheet name="Bank system" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
   <si>
     <t>Feature</t>
   </si>
@@ -54,9 +55,6 @@
     <t>Change PIN</t>
   </si>
   <si>
-    <t>Mini Statement</t>
-  </si>
-  <si>
     <t>Receipt</t>
   </si>
   <si>
@@ -103,13 +101,106 @@
   </si>
   <si>
     <t>Allow the user to cancel a transaction before it is completed</t>
+  </si>
+  <si>
+    <t>Navigation (main menu)</t>
+  </si>
+  <si>
+    <t>Display after validation of the PIN. Allow the user selects options in ATM</t>
+  </si>
+  <si>
+    <t>Transaction Processing</t>
+  </si>
+  <si>
+    <t>Withdrawl Processing</t>
+  </si>
+  <si>
+    <t>Deposit Processing</t>
+  </si>
+  <si>
+    <t>Transaction History</t>
+  </si>
+  <si>
+    <t>Account Authentication</t>
+  </si>
+  <si>
+    <t>Account Management</t>
+  </si>
+  <si>
+    <t>Balance Management</t>
+  </si>
+  <si>
+    <t>Verify the user's account/PIN when required</t>
+  </si>
+  <si>
+    <t>Manage user account information and status</t>
+  </si>
+  <si>
+    <t>Store and update the customer's account balance</t>
+  </si>
+  <si>
+    <t>Process transactions and received from the ATM</t>
+  </si>
+  <si>
+    <t>Deduct the withdrawn amount from the user's account</t>
+  </si>
+  <si>
+    <t>Add the deposited amount the user's account</t>
+  </si>
+  <si>
+    <t>Provide the latest account balance to the ATM</t>
+  </si>
+  <si>
+    <t>Record completed transactions for the account</t>
+  </si>
+  <si>
+    <t>Need confirm</t>
+  </si>
+  <si>
+    <t>REQ-1</t>
+  </si>
+  <si>
+    <t>REQ-2</t>
+  </si>
+  <si>
+    <t>REQ-3</t>
+  </si>
+  <si>
+    <t>REQ-4</t>
+  </si>
+  <si>
+    <t>REQ-5</t>
+  </si>
+  <si>
+    <t>REQ-6</t>
+  </si>
+  <si>
+    <t>REQ-7</t>
+  </si>
+  <si>
+    <t>REQ-8</t>
+  </si>
+  <si>
+    <t>REQ-9</t>
+  </si>
+  <si>
+    <t>REQ-10</t>
+  </si>
+  <si>
+    <t>REQ-11</t>
+  </si>
+  <si>
+    <t>REQ-12</t>
+  </si>
+  <si>
+    <t>REQ-13</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,6 +212,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -146,13 +243,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -434,120 +534,260 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24" style="2" customWidth="1"/>
-    <col min="2" max="2" width="55.7265625" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="8.7265625" style="2"/>
+    <col min="1" max="1" width="13.08984375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="26.26953125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="53.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.26953125" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="2" t="s">
+    <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="2" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="2" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="2" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+    <row r="13" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>14</v>
+      <c r="C14" s="2" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D76FD108-D374-497F-925F-3F73DFCAD246}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24.90625" customWidth="1"/>
+    <col min="2" max="2" width="52.36328125" customWidth="1"/>
+    <col min="3" max="3" width="39.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Format file Feature as default when open it
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Feature.xlsx
+++ b/C/Project/ATM_Sim/Doc/Feature.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BF85B32-D4AA-4139-BEE5-D6FD82369E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE50E53C-46D6-416D-A5D3-26DCE320D31E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ATM" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Removed ID requirement as request
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Feature.xlsx
+++ b/C/Project/ATM_Sim/Doc/Feature.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE50E53C-46D6-416D-A5D3-26DCE320D31E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29057757-9F6A-49F9-8C0E-D6195AF002ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="43">
   <si>
     <t>Feature</t>
   </si>
@@ -155,45 +155,6 @@
   </si>
   <si>
     <t>Need confirm</t>
-  </si>
-  <si>
-    <t>REQ-1</t>
-  </si>
-  <si>
-    <t>REQ-2</t>
-  </si>
-  <si>
-    <t>REQ-3</t>
-  </si>
-  <si>
-    <t>REQ-4</t>
-  </si>
-  <si>
-    <t>REQ-5</t>
-  </si>
-  <si>
-    <t>REQ-6</t>
-  </si>
-  <si>
-    <t>REQ-7</t>
-  </si>
-  <si>
-    <t>REQ-8</t>
-  </si>
-  <si>
-    <t>REQ-9</t>
-  </si>
-  <si>
-    <t>REQ-10</t>
-  </si>
-  <si>
-    <t>REQ-11</t>
-  </si>
-  <si>
-    <t>REQ-12</t>
-  </si>
-  <si>
-    <t>REQ-13</t>
   </si>
 </sst>
 </file>
@@ -534,164 +495,124 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.08984375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="26.26953125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="53.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.26953125" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="2"/>
+    <col min="1" max="1" width="26.26953125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="53.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.26953125" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>44</v>
+        <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="2" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>